<commit_message>
[DataDriven] 데이터 드리븐 버그 임시 공사     20260521
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/0_DateDialogue.xlsx
+++ b/JsonConverter/ExcelFiles/0_DateDialogue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0_SonghaUnityGame\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE72CE29-658C-474D-B075-0BA82D07DA74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F9B784B-C56E-4071-9AF5-9D561D77922E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6375" yWindow="1050" windowWidth="15465" windowHeight="14055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2730" yWindow="1740" windowWidth="23505" windowHeight="14460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DNTable_Weapon" sheetId="1" r:id="rId1"/>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
-  <si>
-    <t>SelectionNameList</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>CharacterDataId</t>
   </si>
@@ -63,12 +60,24 @@
     <t>(name)</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
+  <si>
+    <t>string</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>NextDialogueId</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>mindDialogue_Opening_1_1_99</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -93,6 +102,12 @@
       <name val="돋움"/>
       <family val="3"/>
       <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -162,7 +177,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -185,6 +200,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -602,7 +618,7 @@
   <dimension ref="A1:G1000"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="1" max="1" width="35.85546875" customWidth="1"/>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="77.140625" customWidth="1"/>
     <col min="5" max="6" width="50.7109375" customWidth="1"/>
@@ -610,7 +626,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -620,56 +636,59 @@
     </row>
     <row r="2" spans="1:7" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>9</v>
+      <c r="C4" s="10" t="s">
+        <v>14</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>

</xml_diff>